<commit_message>
Adds sql-connection to store experiment-data
</commit_message>
<xml_diff>
--- a/resources/protocols/G0241_19_C.xlsx
+++ b/resources/protocols/G0241_19_C.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="headers" sheetId="1" state="visible" r:id="rId2"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="121">
   <si>
     <t xml:space="preserve">Header name</t>
   </si>
@@ -153,7 +153,7 @@
     <t xml:space="preserve">(?i)(?:^(L\s*(?:0225\/15)?)[\s,]*)</t>
   </si>
   <si>
-    <t xml:space="preserve">Procedure name</t>
+    <t xml:space="preserve">name</t>
   </si>
   <si>
     <t xml:space="preserve">allowed</t>
@@ -210,10 +210,7 @@
     <t xml:space="preserve">cannula implant</t>
   </si>
   <si>
-    <t xml:space="preserve">Drug name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">default_amount</t>
+    <t xml:space="preserve">amount</t>
   </si>
   <si>
     <t xml:space="preserve">days_after_surgery</t>
@@ -999,27 +996,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>42</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>64</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>65</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>47</v>
@@ -1028,15 +1025,15 @@
         <v>0</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>68</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>47</v>
@@ -1045,15 +1042,15 @@
         <v>0</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>47</v>
@@ -1062,15 +1059,15 @@
         <v>3</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>47</v>
@@ -1079,32 +1076,32 @@
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>49</v>
@@ -1139,12 +1136,12 @@
         <v>42</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>47</v>
@@ -1181,27 +1178,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1229,7 +1226,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -1237,26 +1234,26 @@
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1283,34 +1280,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1318,7 +1315,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1342,59 +1339,59 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>105</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>109</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1402,30 +1399,30 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>118</v>
-      </c>
       <c r="E8" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>